<commit_message>
New update to solve issue with the template was published
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF252158-D943-4D1F-8229-28EB981564C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Transaction</t>
   </si>
@@ -43,55 +43,7 @@
     <t>ejecutar</t>
   </si>
   <si>
-    <t>ZMM026</t>
-  </si>
-  <si>
-    <t>disposicion</t>
-  </si>
-  <si>
-    <t>LX02</t>
-  </si>
-  <si>
-    <t>COHV</t>
-  </si>
-  <si>
-    <t>checks</t>
-  </si>
-  <si>
-    <t>ZCO017</t>
-  </si>
-  <si>
-    <t>ZPP029_1</t>
-  </si>
-  <si>
-    <t>BOM</t>
-  </si>
-  <si>
-    <t>MB52</t>
-  </si>
-  <si>
-    <t>ZSD053</t>
-  </si>
-  <si>
-    <t>LT23</t>
-  </si>
-  <si>
-    <t>VL06O</t>
-  </si>
-  <si>
-    <t>listas sal</t>
-  </si>
-  <si>
-    <t>vista posicion</t>
-  </si>
-  <si>
-    <t>ODM</t>
-  </si>
-  <si>
     <t>Step4</t>
-  </si>
-  <si>
-    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -581,8 +533,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -938,7 +891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -955,11 +908,11 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
@@ -969,119 +922,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New version with all SAP transacions was published
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF252158-D943-4D1F-8229-28EB981564C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
   <si>
     <t>Transaction</t>
   </si>
@@ -43,7 +43,55 @@
     <t>ejecutar</t>
   </si>
   <si>
+    <t>ZMM026</t>
+  </si>
+  <si>
+    <t>disposicion</t>
+  </si>
+  <si>
+    <t>LX02</t>
+  </si>
+  <si>
+    <t>COHV</t>
+  </si>
+  <si>
+    <t>checks</t>
+  </si>
+  <si>
+    <t>ZCO017</t>
+  </si>
+  <si>
+    <t>ZPP029_1</t>
+  </si>
+  <si>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>MB52</t>
+  </si>
+  <si>
+    <t>ZSD053</t>
+  </si>
+  <si>
+    <t>LT23</t>
+  </si>
+  <si>
+    <t>VL06O</t>
+  </si>
+  <si>
+    <t>listas sal</t>
+  </si>
+  <si>
+    <t>vista posicion</t>
+  </si>
+  <si>
+    <t>ODM</t>
+  </si>
+  <si>
     <t>Step4</t>
+  </si>
+  <si>
+    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -533,9 +581,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -891,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -908,11 +955,11 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
@@ -920,6 +967,119 @@
       </c>
       <c r="C2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TransactionSap file was restore, same version was published
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF16B7A-DE55-40F5-A275-AB9F706CD4FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
   <si>
     <t>Transaction</t>
   </si>
@@ -34,19 +34,64 @@
     <t>Step3</t>
   </si>
   <si>
+    <t>ZMG002_01</t>
+  </si>
+  <si>
+    <t>variante</t>
+  </si>
+  <si>
     <t>ejecutar</t>
   </si>
   <si>
+    <t>ZMM026</t>
+  </si>
+  <si>
+    <t>disposicion</t>
+  </si>
+  <si>
+    <t>LX02</t>
+  </si>
+  <si>
+    <t>COHV</t>
+  </si>
+  <si>
+    <t>checks</t>
+  </si>
+  <si>
+    <t>ZCO017</t>
+  </si>
+  <si>
+    <t>ZPP029_1</t>
+  </si>
+  <si>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>MB52</t>
+  </si>
+  <si>
+    <t>ZSD053</t>
+  </si>
+  <si>
+    <t>LT23</t>
+  </si>
+  <si>
+    <t>VL06O</t>
+  </si>
+  <si>
+    <t>listas sal</t>
+  </si>
+  <si>
+    <t>vista posicion</t>
+  </si>
+  <si>
+    <t>ODM</t>
+  </si>
+  <si>
     <t>Step4</t>
   </si>
   <si>
-    <t>COHV</t>
-  </si>
-  <si>
-    <t>checks</t>
-  </si>
-  <si>
-    <t>disposicion</t>
+    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -536,9 +581,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -894,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -911,21 +955,131 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to solving issue in SAP for transaction ZPP029_1 were done, new version published
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511B9735-C692-444B-AEC7-3A1E6781154F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Transaction</t>
   </si>
@@ -34,64 +34,13 @@
     <t>Step3</t>
   </si>
   <si>
-    <t>ZMG002_01</t>
-  </si>
-  <si>
-    <t>variante</t>
-  </si>
-  <si>
-    <t>ejecutar</t>
-  </si>
-  <si>
-    <t>ZMM026</t>
-  </si>
-  <si>
-    <t>disposicion</t>
-  </si>
-  <si>
-    <t>LX02</t>
-  </si>
-  <si>
-    <t>COHV</t>
-  </si>
-  <si>
-    <t>checks</t>
-  </si>
-  <si>
-    <t>ZCO017</t>
+    <t>Step4</t>
   </si>
   <si>
     <t>ZPP029_1</t>
   </si>
   <si>
     <t>BOM</t>
-  </si>
-  <si>
-    <t>MB52</t>
-  </si>
-  <si>
-    <t>ZSD053</t>
-  </si>
-  <si>
-    <t>LT23</t>
-  </si>
-  <si>
-    <t>VL06O</t>
-  </si>
-  <si>
-    <t>listas sal</t>
-  </si>
-  <si>
-    <t>vista posicion</t>
-  </si>
-  <si>
-    <t>ODM</t>
-  </si>
-  <si>
-    <t>Step4</t>
-  </si>
-  <si>
-    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -938,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -955,131 +904,15 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Same version with the transactions file restored
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511B9735-C692-444B-AEC7-3A1E6781154F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
   <si>
     <t>Transaction</t>
   </si>
@@ -34,13 +34,64 @@
     <t>Step3</t>
   </si>
   <si>
+    <t>ZMG002_01</t>
+  </si>
+  <si>
+    <t>variante</t>
+  </si>
+  <si>
+    <t>ejecutar</t>
+  </si>
+  <si>
+    <t>ZMM026</t>
+  </si>
+  <si>
+    <t>disposicion</t>
+  </si>
+  <si>
+    <t>LX02</t>
+  </si>
+  <si>
+    <t>COHV</t>
+  </si>
+  <si>
+    <t>checks</t>
+  </si>
+  <si>
+    <t>ZCO017</t>
+  </si>
+  <si>
+    <t>ZPP029_1</t>
+  </si>
+  <si>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>MB52</t>
+  </si>
+  <si>
+    <t>ZSD053</t>
+  </si>
+  <si>
+    <t>LT23</t>
+  </si>
+  <si>
+    <t>VL06O</t>
+  </si>
+  <si>
+    <t>listas sal</t>
+  </si>
+  <si>
+    <t>vista posicion</t>
+  </si>
+  <si>
+    <t>ODM</t>
+  </si>
+  <si>
     <t>Step4</t>
   </si>
   <si>
-    <t>ZPP029_1</t>
-  </si>
-  <si>
-    <t>BOM</t>
+    <t>filtrar pedido</t>
   </si>
 </sst>
 </file>
@@ -887,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -904,15 +955,131 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
select disposition to transaction VÑ06o was added, the macro script was updated
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5A05C-60BD-4EC1-A074-DCA3DDA413D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF3B7FF-D415-4EBD-B1B7-160BEFE6F6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>Transaction</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>filtrar pedido</t>
+  </si>
+  <si>
+    <t>Step5</t>
   </si>
 </sst>
 </file>
@@ -938,10 +941,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -957,8 +960,11 @@
       <c r="E1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -969,7 +975,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -980,7 +986,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -991,7 +997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1005,7 +1011,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1016,7 +1022,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1024,7 +1030,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1035,7 +1041,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1049,7 +1055,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1060,7 +1066,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1076,8 +1082,11 @@
       <c r="E11" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
New version was pblished
</commit_message>
<xml_diff>
--- a/Data/Input/TransaccionesSAP.xlsx
+++ b/Data/Input/TransaccionesSAP.xlsx
@@ -8,32 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA61633-FBCE-4085-8E6D-C4EF02F3D25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAA896F-CE2B-49AF-A793-F0DF29802429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E7D37262-4DB0-4AD2-A290-68AC6299F871}"/>
   </bookViews>
   <sheets>
     <sheet name="TransaccionesSAP" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>Transaction</t>
   </si>
@@ -47,13 +34,67 @@
     <t>Step3</t>
   </si>
   <si>
+    <t>ZMG002_01</t>
+  </si>
+  <si>
+    <t>variante</t>
+  </si>
+  <si>
+    <t>ejecutar</t>
+  </si>
+  <si>
+    <t>ZMM026</t>
+  </si>
+  <si>
+    <t>disposicion</t>
+  </si>
+  <si>
+    <t>LX02</t>
+  </si>
+  <si>
+    <t>COHV</t>
+  </si>
+  <si>
+    <t>checks</t>
+  </si>
+  <si>
+    <t>ZCO017</t>
+  </si>
+  <si>
+    <t>ZPP029_1</t>
+  </si>
+  <si>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>MB52</t>
+  </si>
+  <si>
+    <t>ZSD053</t>
+  </si>
+  <si>
+    <t>LT23</t>
+  </si>
+  <si>
+    <t>VL06O</t>
+  </si>
+  <si>
+    <t>listas sal</t>
+  </si>
+  <si>
+    <t>vista posicion</t>
+  </si>
+  <si>
+    <t>ODM</t>
+  </si>
+  <si>
     <t>Step4</t>
   </si>
   <si>
+    <t>filtrar pedido</t>
+  </si>
+  <si>
     <t>Step5</t>
-  </si>
-  <si>
-    <t>ODM</t>
   </si>
 </sst>
 </file>
@@ -900,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1487AD3F-8DFF-47B2-8A8A-A4855C7319A0}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -917,15 +958,137 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>